<commit_message>
Bulk import: 4 magazine articles on the approved article template
- urls-article.txt: arctic-surfing, guide-la-skateparks, san-diego-surf,
  ski-touring (plus western-australia, re-imported unchanged)
- wknd-article: the sidebar download component (LA skateparks PDF) becomes
  default content: description, file details and a bold link (primary
  button); the title link repeats the button and is dropped
- wknd-cleanup alt rule: after the nearest heading, empty alts fall back to
  a descriptive file name (surfer-wave-02.jpeg -> "Surfer wave"), then the
  page title (hero images above the h1). All fallbacks stay in altReview.
- upload-to-da.mjs: linked PDFs are uploaded to /assets/<page>/, previewed
  and linked site-relative
- bundles and reports rebuilt; home, magazine and western-australia
  re-import byte-identical

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article.report.xlsx
+++ b/tools/importer/reports/import-article.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="57">
   <si>
     <t>_reportFile</t>
   </si>
@@ -58,7 +58,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-25T13:04:00.262Z</t>
+    <t>2026-09-27T17:14:23.734Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -82,7 +82,7 @@
     <t>magazine</t>
   </si>
   <si>
-    <t>2026-09-27T14:31:04.891Z</t>
+    <t>2026-09-27T17:14:29.373Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -91,22 +91,91 @@
     <t>https://wknd.site/us/en/magazine.html</t>
   </si>
   <si>
+    <t>us/en/magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
+    <t>["Surfer back from the ocean — empty alt, used file name","Aloha Spirits in Northern Norway — empty alt, used nearest heading","Clear skies — empty alt, used nearest heading","Mythical northern lights — empty alt, used nearest heading"]</t>
+  </si>
+  <si>
+    <t>["columns-author","cards-related"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing</t>
+  </si>
+  <si>
+    <t>article</t>
+  </si>
+  <si>
+    <t>2026-09-27T17:14:39.932Z</t>
+  </si>
+  <si>
+    <t>Arctic Surfing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>["Venice Beach Skatepark — empty alt, used nearest heading"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>2026-09-27T17:14:46.011Z</t>
+  </si>
+  <si>
+    <t>Ultimate Guide to LA Skateparks</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/guide-la-skateparks.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf</t>
+  </si>
+  <si>
+    <t>2026-09-27T17:14:51.948Z</t>
+  </si>
+  <si>
+    <t>San Diego Surf Spots</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/san-diego-surf.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>["Ski Touring — empty alt, used page title","Ski Touring (image 2) — empty alt, used nearest heading","Ski Touring (image 3) — empty alt, used nearest heading","Ski Touring (image 4) — empty alt, used nearest heading","Ski Touring (image 5) — empty alt, used nearest heading"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-09-27T17:14:56.103Z</t>
+  </si>
+  <si>
+    <t>Ski Touring</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/ski-touring.html</t>
+  </si>
+  <si>
     <t>us/en/magazine/western-australia.report.json</t>
   </si>
   <si>
     <t>["Hiking and camping on the coast — empty alt, used nearest heading","A trusty vehicle — empty alt, used nearest heading","Surfing is a must do — empty alt, used nearest heading"]</t>
   </si>
   <si>
-    <t>["columns-author","cards-related"]</t>
-  </si>
-  <si>
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>article</t>
-  </si>
-  <si>
-    <t>2026-09-27T15:18:17.504Z</t>
+    <t>2026-09-27T17:14:34.225Z</t>
   </si>
   <si>
     <t>Western Australia</t>
@@ -501,15 +570,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="46" customWidth="1"/>
+    <col min="1" max="1" width="48" customWidth="1"/>
     <col min="2" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="8" max="8" width="33" customWidth="1"/>
     <col min="9" max="9" width="50" customWidth="1"/>
   </cols>
   <sheetData>
@@ -627,6 +696,122 @@
       </c>
       <c r="I4" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H7" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Articles: plain-text quotes, rich-text headings, sidebar download styling
Critique fixes for the bulk-imported articles:
- wknd-article: a quotation inside ordinary text (arctic surfing) becomes
  paragraphs; only the quote component stays a boxed blockquote
- wknd-article: when every body h2 is rich text (san diego surf), the body
  section gets the "plain-headings" style: no underline, text-wide, the
  text's 27px heading gap (title-component headings are unchanged)
- download: keeps the source's label as a plain h3 (no second PDF link)
- styles.css: sidebar download label/description/details spacing as the
  WKND components, dark button with the WKND download icon; the article
  text's 14px outset no longer applies to sidebar paragraphs
- icons/download.svg from the WKND icon font (e907)

western-australia re-imports byte-identical.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article.report.xlsx
+++ b/tools/importer/reports/import-article.report.xlsx
@@ -106,7 +106,7 @@
     <t>article</t>
   </si>
   <si>
-    <t>2026-09-27T17:14:39.932Z</t>
+    <t>2026-09-27T17:24:48.053Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -124,7 +124,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-27T17:14:46.011Z</t>
+    <t>2026-09-27T17:24:52.713Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -139,7 +139,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-27T17:14:51.948Z</t>
+    <t>2026-09-27T17:24:58.811Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -157,7 +157,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-27T17:14:56.103Z</t>
+    <t>2026-09-27T17:25:03.914Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -175,7 +175,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-27T17:14:34.225Z</t>
+    <t>2026-09-27T17:24:42.179Z</t>
   </si>
   <si>
     <t>Western Australia</t>

</xml_diff>

<commit_message>
Articles: image captions, text-wide rich-text headings keep the article gap
- wknd-article: an image's caption (WKND image title, shown under the
  image) becomes an italic paragraph after it instead of loose text
  inside the image paragraph (san diego surf)
- styles.css: that paragraph is styled as the WKND caption (14px/21px
  semibold uppercase, 11px under the image); italic + bold address lines
  are excluded
- plain-headings keeps the article's 40.5px heading gap, as measured on
  the source; only the underline and the width differ

western-australia re-imports byte-identical.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article.report.xlsx
+++ b/tools/importer/reports/import-article.report.xlsx
@@ -106,7 +106,7 @@
     <t>article</t>
   </si>
   <si>
-    <t>2026-09-27T17:24:48.053Z</t>
+    <t>2026-09-27T17:31:08.046Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -124,7 +124,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-27T17:24:52.713Z</t>
+    <t>2026-09-27T17:31:13.045Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -139,7 +139,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-27T17:24:58.811Z</t>
+    <t>2026-09-27T17:31:20.736Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -157,7 +157,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-27T17:25:03.914Z</t>
+    <t>2026-09-27T17:31:26.818Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -175,7 +175,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-27T17:24:42.179Z</t>
+    <t>2026-09-27T17:31:02.849Z</t>
   </si>
   <si>
     <t>Western Australia</t>

</xml_diff>

<commit_message>
Quotes: single-paragraph quotations stay blockquotes, set in the running text
A quote followed by its attribution/definition paragraph(s) is the pull
quote (grey box, serif, accent underline; western australia, LA, ski
touring). A one-paragraph quotation inside ordinary text (arctic surfing)
keeps its blockquote semantics and is set as on wknd.site: text-wide,
18px/27px, 18px margins. Replaces unwrapping it into a paragraph.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article.report.xlsx
+++ b/tools/importer/reports/import-article.report.xlsx
@@ -106,7 +106,7 @@
     <t>article</t>
   </si>
   <si>
-    <t>2026-09-27T17:31:08.046Z</t>
+    <t>2026-09-27T17:57:34.382Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -124,7 +124,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-27T17:31:13.045Z</t>
+    <t>2026-09-27T17:57:42.113Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -139,7 +139,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-27T17:31:20.736Z</t>
+    <t>2026-09-27T17:57:47.754Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -157,7 +157,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-27T17:31:26.818Z</t>
+    <t>2026-09-27T17:57:53.581Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -175,7 +175,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-27T17:31:02.849Z</t>
+    <t>2026-09-27T17:57:29.061Z</t>
   </si>
   <si>
     <t>Western Australia</t>

</xml_diff>